<commit_message>
add BU03 module information
</commit_message>
<xml_diff>
--- a/BU03_info/BU03_data_calibration.xlsx
+++ b/BU03_info/BU03_data_calibration.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NTU\車車課\Light_Tracker\BU03_info\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1AFC3B9-F8F1-48C7-94E2-28A802B6FD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView xWindow="28635" yWindow="-165" windowWidth="29130" windowHeight="15810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Raw Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>UWB Display Distance（mm）</t>
   </si>
@@ -46,179 +53,98 @@
   <si>
     <t>Difference</t>
   </si>
+  <si>
+    <t>30cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>45cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>60cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>75cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>90cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>105cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>120cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>135cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>150cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>165cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>180cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>195cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>210cm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="180" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="新細明體"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="5" tint="-0.249977111117893"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
+      <name val="新細明體"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -227,198 +153,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="3" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -485,338 +231,47 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="zh-CN"/>
+  <c:lang val="zh-TW"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -847,6 +302,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Actual </a:t>
             </a:r>
             <a:r>
@@ -854,6 +310,7 @@
               <a:t>D</a:t>
             </a:r>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>istance（Self-measurement</a:t>
             </a:r>
             <a:r>
@@ -861,12 +318,12 @@
               <a:t> </a:t>
             </a:r>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>mm）</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -875,6 +332,26 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr defTabSz="914400">
+            <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-TW"/>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -954,6 +431,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="zh-TW"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -975,22 +453,7 @@
                     <a:noFill/>
                   </a:ln>
                 </c15:spPr>
-                <c15:layout/>
                 <c15:showLeaderLines val="0"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -1011,7 +474,7 @@
               <c:layout>
                 <c:manualLayout>
                   <c:x val="-0.478820690096665"/>
-                  <c:y val="-0.00104535034386524"/>
+                  <c:y val="-1.0453503438652399E-3"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
@@ -1039,6 +502,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
+                  <a:endParaRPr lang="zh-TW"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -1049,6 +513,45 @@
               <c:numCache>
                 <c:formatCode>0.00_);[Red]\(0.00\)</c:formatCode>
                 <c:ptCount val="36"/>
+                <c:pt idx="0">
+                  <c:v>534.70100000000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>691.35900000000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>812.83900000000006</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>943.7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1206.3599999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1322.68</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1643.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1965.73</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1909.91</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2035.62</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2113.4699999999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2410.37</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2511.2199999999998</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1058,10 +561,54 @@
               <c:numCache>
                 <c:formatCode>0.00_);[Red]\(0.00\)</c:formatCode>
                 <c:ptCount val="36"/>
+                <c:pt idx="0">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>450</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>750</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1050</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1650</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1800</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1950</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2100</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-7706-42AA-9770-8DCD4B7C371D}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -1115,12 +662,12 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>UWB Display Distance</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1129,6 +676,26 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr defTabSz="914400">
+                <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="zh-TW"/>
+            </a:p>
+          </c:txPr>
         </c:title>
         <c:numFmt formatCode="0.00_);[Red]\(0.00\)" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1164,6 +731,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="481425184"/>
@@ -1211,12 +779,12 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>Actual Distance</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1225,6 +793,26 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr defTabSz="914400">
+                <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="zh-TW"/>
+            </a:p>
+          </c:txPr>
         </c:title>
         <c:numFmt formatCode="0.00_);[Red]\(0.00\)" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1260,6 +848,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="481428136"/>
@@ -1305,6 +894,7 @@
       <a:pPr>
         <a:defRPr lang="zh-CN"/>
       </a:pPr>
+      <a:endParaRPr lang="zh-TW"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1872,7 +1462,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -1886,14 +1476,20 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>40005</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="图表 1"/>
+        <xdr:cNvPr id="2" name="图表 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8790940" y="0"/>
-        <a:ext cx="12251055" cy="4564380"/>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2158,2115 +1754,2763 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G345"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6666666666667" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.775" style="2" customWidth="1"/>
+    <col min="1" max="1" width="27.59765625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.69921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.796875" style="2" customWidth="1"/>
     <col min="4" max="4" width="31" style="3" customWidth="1"/>
-    <col min="5" max="5" width="15.775" customWidth="1"/>
+    <col min="5" max="5" width="15.796875" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="21.5583333333333" customWidth="1"/>
-    <col min="17" max="17" width="9.10833333333333" customWidth="1"/>
+    <col min="7" max="7" width="21.59765625" customWidth="1"/>
+    <col min="17" max="17" width="9.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="3:3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>534.70100000000002</v>
+      </c>
+      <c r="B2" s="1">
+        <v>300</v>
+      </c>
       <c r="C2" s="2">
-        <f t="shared" ref="C2:C17" si="0">A2-B2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="3:3">
+        <f>A2-B2</f>
+        <v>234.70100000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>691.35900000000004</v>
+      </c>
+      <c r="B3" s="1">
+        <v>450</v>
+      </c>
       <c r="C3" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="3:3">
+        <f>A3-B3</f>
+        <v>241.35900000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>812.83900000000006</v>
+      </c>
+      <c r="B4" s="1">
+        <v>600</v>
+      </c>
       <c r="C4" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="3:3">
+        <f>A4-B4</f>
+        <v>212.83900000000006</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>943.7</v>
+      </c>
+      <c r="B5" s="1">
+        <v>750</v>
+      </c>
       <c r="C5" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="3:3">
+        <f>A5-B5</f>
+        <v>193.70000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1206.3599999999999</v>
+      </c>
+      <c r="B6" s="1">
+        <v>900</v>
+      </c>
       <c r="C6" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="3:3">
+        <f>A6-B6</f>
+        <v>306.3599999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1322.68</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1050</v>
+      </c>
       <c r="C7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="3:3">
+        <f>A7-B7</f>
+        <v>272.68000000000006</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1643.5</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1200</v>
+      </c>
       <c r="C8" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="3:3">
+        <f>A8-B8</f>
+        <v>443.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1965.73</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1350</v>
+      </c>
       <c r="C9" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="3:3">
+        <f>A9-B9</f>
+        <v>615.73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1909.91</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1500</v>
+      </c>
       <c r="C10" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="3:3">
+        <f>A10-B10</f>
+        <v>409.91000000000008</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>2035.62</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1650</v>
+      </c>
       <c r="C11" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="3:3">
+        <f>A11-B11</f>
+        <v>385.61999999999989</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>2113.4699999999998</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1800</v>
+      </c>
       <c r="C12" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="3:3">
+        <f>A12-B12</f>
+        <v>313.4699999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>2410.37</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1950</v>
+      </c>
       <c r="C13" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="3:3">
+        <f>A13-B13</f>
+        <v>460.36999999999989</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>2511.2199999999998</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2100</v>
+      </c>
       <c r="C14" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="3:3">
+        <f>A14-B14</f>
+        <v>411.2199999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C15" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="3:3">
+        <f>A15-B15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C16" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="3:3">
+        <f t="shared" ref="C16:C17" si="0">A16-B16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C17" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="3:3">
+    <row r="18" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C18" s="2">
         <f t="shared" ref="C18:C65" si="1">A18-B18</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:3">
+    <row r="19" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C19" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="3:3">
+    <row r="20" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C20" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="3:3">
+    <row r="21" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C21" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:3">
+    <row r="22" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C22" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:3">
+    <row r="23" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C23" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:3">
+    <row r="24" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C24" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:3">
+    <row r="25" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C25" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="15" spans="3:3">
+    <row r="26" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C26" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:7">
+    <row r="27" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C27" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="7" t="s">
+      <c r="F27" s="4"/>
+      <c r="G27" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" ht="15" spans="3:7">
+    <row r="28" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C28" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="9" t="s">
+      <c r="F28" s="6"/>
+      <c r="G28" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="3:3">
+    <row r="29" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C29" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:3">
+    <row r="30" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C30" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:3">
+    <row r="31" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C31" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="3:3">
+    <row r="32" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C32" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C33" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:3">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C34" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:3">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C35" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="3:3">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C36" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="3:3">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C37" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="3:3">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C38" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="3:3">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C39" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="3:3">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C40" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="3:3">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C41" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="3:3">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C42" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="3:3">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C43" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="3:3">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C44" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:3">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C45" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="3:3">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C46" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="3:3">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C47" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="3:3">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C48" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:3">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C49" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:3">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C50" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:3">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C51" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="3:3">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C52" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="3:3">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C53" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="3:3">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C54" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="3:3">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C55" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="3:3">
+    <row r="56" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C56" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="3:3">
+    <row r="57" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C57" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="3:3">
+    <row r="58" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C58" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="3:3">
+    <row r="59" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C59" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="3:3">
+    <row r="60" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C60" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="3:3">
+    <row r="61" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C61" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="3:3">
+    <row r="62" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C62" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="3:3">
+    <row r="63" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C63" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="3:3">
+    <row r="64" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C64" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="3:3">
+    <row r="65" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C65" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="3:3">
+    <row r="66" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C66" s="2">
         <f t="shared" ref="C66:C129" si="2">A66-B66</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="3:3">
+    <row r="67" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C67" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="3:3">
+    <row r="68" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C68" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="3:3">
+    <row r="69" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C69" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="3:3">
+    <row r="70" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C70" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="3:3">
+    <row r="71" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C71" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="3:3">
+    <row r="72" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C72" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="3:3">
+    <row r="73" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C73" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="3:3">
+    <row r="74" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C74" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="3:3">
+    <row r="75" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C75" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="3:3">
+    <row r="76" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C76" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="3:3">
+    <row r="77" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C77" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="3:3">
+    <row r="78" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C78" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="3:3">
+    <row r="79" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C79" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="3:3">
+    <row r="80" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C80" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="3:3">
+    <row r="81" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C81" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="3:3">
+    <row r="82" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C82" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="3:3">
+    <row r="83" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C83" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="3:3">
+    <row r="84" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C84" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="3:3">
+    <row r="85" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C85" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="3:3">
+    <row r="86" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C86" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="3:3">
+    <row r="87" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C87" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="3:3">
+    <row r="88" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C88" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="3:3">
+    <row r="89" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C89" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="3:3">
+    <row r="90" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C90" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="3:3">
+    <row r="91" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C91" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="3:3">
+    <row r="92" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C92" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="3:3">
+    <row r="93" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C93" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="3:3">
+    <row r="94" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C94" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="3:3">
+    <row r="95" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C95" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="3:3">
+    <row r="96" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C96" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="3:3">
+    <row r="97" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C97" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="3:3">
+    <row r="98" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C98" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="3:3">
+    <row r="99" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C99" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="3:3">
+    <row r="100" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C100" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="3:3">
+    <row r="101" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C101" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="3:3">
+    <row r="102" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C102" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="3:3">
+    <row r="103" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C103" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="3:3">
+    <row r="104" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C104" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="3:3">
+    <row r="105" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C105" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="3:3">
+    <row r="106" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C106" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="3:3">
+    <row r="107" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C107" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="3:3">
+    <row r="108" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C108" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="3:3">
+    <row r="109" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C109" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="3:3">
+    <row r="110" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C110" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="3:3">
+    <row r="111" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C111" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="3:3">
+    <row r="112" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C112" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="3:3">
+    <row r="113" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C113" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="3:3">
+    <row r="114" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C114" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="3:3">
+    <row r="115" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C115" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="3:3">
+    <row r="116" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C116" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="3:3">
+    <row r="117" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C117" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="3:3">
+    <row r="118" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C118" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="3:3">
+    <row r="119" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C119" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="3:3">
+    <row r="120" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C120" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="3:3">
+    <row r="121" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C121" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="3:3">
+    <row r="122" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C122" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="3:3">
+    <row r="123" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C123" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="3:3">
+    <row r="124" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C124" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="3:3">
+    <row r="125" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C125" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="3:3">
+    <row r="126" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C126" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="3:3">
+    <row r="127" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C127" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="3:3">
+    <row r="128" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C128" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="3:3">
+    <row r="129" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C129" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="3:3">
+    <row r="130" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C130" s="2">
         <f t="shared" ref="C130:C193" si="3">A130-B130</f>
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="3:3">
+    <row r="131" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C131" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="3:3">
+    <row r="132" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C132" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="3:3">
+    <row r="133" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C133" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="3:3">
+    <row r="134" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C134" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="3:3">
+    <row r="135" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C135" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="3:3">
+    <row r="136" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C136" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="3:3">
+    <row r="137" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C137" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="3:3">
+    <row r="138" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C138" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="3:3">
+    <row r="139" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C139" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="3:3">
+    <row r="140" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C140" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="3:3">
+    <row r="141" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C141" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="3:3">
+    <row r="142" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C142" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="3:3">
+    <row r="143" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C143" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="3:3">
+    <row r="144" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C144" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="3:3">
+    <row r="145" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C145" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="3:3">
+    <row r="146" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C146" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="3:3">
+    <row r="147" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C147" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="3:3">
+    <row r="148" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C148" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="3:3">
+    <row r="149" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C149" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="3:3">
+    <row r="150" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C150" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="3:3">
+    <row r="151" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C151" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="3:3">
+    <row r="152" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C152" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="3:3">
+    <row r="153" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C153" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="3:3">
+    <row r="154" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C154" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="3:3">
+    <row r="155" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C155" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="3:3">
+    <row r="156" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C156" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="3:3">
+    <row r="157" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C157" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="3:3">
+    <row r="158" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C158" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="3:3">
+    <row r="159" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C159" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="3:3">
+    <row r="160" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C160" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="3:3">
+    <row r="161" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C161" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="3:3">
+    <row r="162" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C162" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="3:3">
+    <row r="163" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C163" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="3:3">
+    <row r="164" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C164" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="3:3">
+    <row r="165" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C165" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="3:3">
+    <row r="166" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C166" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="3:3">
+    <row r="167" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C167" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="3:3">
+    <row r="168" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C168" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="3:3">
+    <row r="169" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C169" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="3:3">
+    <row r="170" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C170" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="3:3">
+    <row r="171" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C171" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="3:3">
+    <row r="172" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C172" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="3:3">
+    <row r="173" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C173" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="3:3">
+    <row r="174" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C174" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="3:3">
+    <row r="175" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C175" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="3:3">
+    <row r="176" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C176" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="3:3">
+    <row r="177" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C177" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="3:3">
+    <row r="178" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C178" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="3:3">
+    <row r="179" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C179" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="3:3">
+    <row r="180" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C180" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="3:3">
+    <row r="181" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C181" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="3:3">
+    <row r="182" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C182" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="3:3">
+    <row r="183" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C183" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="3:3">
+    <row r="184" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C184" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="3:3">
+    <row r="185" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C185" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="3:3">
+    <row r="186" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C186" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="3:3">
+    <row r="187" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C187" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="3:3">
+    <row r="188" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C188" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="3:3">
+    <row r="189" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C189" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="3:3">
+    <row r="190" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C190" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="3:3">
+    <row r="191" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C191" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="3:3">
+    <row r="192" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C192" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="3:3">
+    <row r="193" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C193" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="3:3">
+    <row r="194" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C194" s="2">
         <f t="shared" ref="C194:C257" si="4">A194-B194</f>
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="3:3">
+    <row r="195" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C195" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="3:3">
+    <row r="196" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C196" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="3:3">
+    <row r="197" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C197" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="3:3">
+    <row r="198" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C198" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="3:3">
+    <row r="199" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C199" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="3:3">
+    <row r="200" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C200" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="3:3">
+    <row r="201" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C201" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="3:3">
+    <row r="202" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C202" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="3:3">
+    <row r="203" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C203" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="3:3">
+    <row r="204" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C204" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="3:3">
+    <row r="205" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C205" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="3:3">
+    <row r="206" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C206" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="3:3">
+    <row r="207" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C207" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="3:3">
+    <row r="208" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C208" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="3:3">
+    <row r="209" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C209" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="3:3">
+    <row r="210" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C210" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="3:3">
+    <row r="211" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C211" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="3:3">
+    <row r="212" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C212" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="3:3">
+    <row r="213" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C213" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="3:3">
+    <row r="214" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C214" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="3:3">
+    <row r="215" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C215" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="3:3">
+    <row r="216" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C216" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="3:3">
+    <row r="217" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C217" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="3:3">
+    <row r="218" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C218" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="3:3">
+    <row r="219" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C219" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="3:3">
+    <row r="220" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C220" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="3:3">
+    <row r="221" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C221" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="3:3">
+    <row r="222" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C222" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="3:3">
+    <row r="223" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C223" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="3:3">
+    <row r="224" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C224" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="3:3">
+    <row r="225" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C225" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="3:3">
+    <row r="226" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C226" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="3:3">
+    <row r="227" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C227" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="3:3">
+    <row r="228" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C228" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="3:3">
+    <row r="229" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C229" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="3:3">
+    <row r="230" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C230" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="3:3">
+    <row r="231" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C231" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="3:3">
+    <row r="232" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C232" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="3:3">
+    <row r="233" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C233" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="3:3">
+    <row r="234" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C234" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="3:3">
+    <row r="235" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C235" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="3:3">
+    <row r="236" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C236" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="3:3">
+    <row r="237" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C237" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="3:3">
+    <row r="238" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C238" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="3:3">
+    <row r="239" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C239" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="3:3">
+    <row r="240" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C240" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="3:3">
+    <row r="241" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C241" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="3:3">
+    <row r="242" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C242" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="3:3">
+    <row r="243" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C243" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="3:3">
+    <row r="244" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C244" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="3:3">
+    <row r="245" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C245" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="3:3">
+    <row r="246" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C246" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="3:3">
+    <row r="247" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C247" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="3:3">
+    <row r="248" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C248" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="3:3">
+    <row r="249" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C249" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="3:3">
+    <row r="250" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C250" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="3:3">
+    <row r="251" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C251" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="3:3">
+    <row r="252" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C252" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="3:3">
+    <row r="253" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C253" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="3:3">
+    <row r="254" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C254" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="3:3">
+    <row r="255" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C255" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="3:3">
+    <row r="256" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C256" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="3:3">
+    <row r="257" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C257" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="3:3">
+    <row r="258" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C258" s="2">
         <f t="shared" ref="C258:C321" si="5">A258-B258</f>
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="3:3">
+    <row r="259" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C259" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="3:3">
+    <row r="260" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C260" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="3:3">
+    <row r="261" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C261" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="3:3">
+    <row r="262" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C262" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="3:3">
+    <row r="263" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C263" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="3:3">
+    <row r="264" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C264" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="3:3">
+    <row r="265" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C265" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="3:3">
+    <row r="266" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C266" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="3:3">
+    <row r="267" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C267" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="3:3">
+    <row r="268" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C268" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="3:3">
+    <row r="269" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C269" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="3:3">
+    <row r="270" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C270" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="3:3">
+    <row r="271" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C271" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="3:3">
+    <row r="272" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C272" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="3:3">
+    <row r="273" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C273" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="3:3">
+    <row r="274" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C274" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="3:3">
+    <row r="275" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C275" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="3:3">
+    <row r="276" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C276" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="3:3">
+    <row r="277" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C277" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="3:3">
+    <row r="278" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C278" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="3:3">
+    <row r="279" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C279" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="3:3">
+    <row r="280" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C280" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="3:3">
+    <row r="281" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C281" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="3:3">
+    <row r="282" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C282" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="3:3">
+    <row r="283" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C283" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="3:3">
+    <row r="284" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C284" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="3:3">
+    <row r="285" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C285" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="3:3">
+    <row r="286" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C286" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="3:3">
+    <row r="287" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C287" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="3:3">
+    <row r="288" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C288" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="3:3">
+    <row r="289" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C289" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="3:3">
+    <row r="290" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C290" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="3:3">
+    <row r="291" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C291" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="3:3">
+    <row r="292" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C292" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="3:3">
+    <row r="293" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C293" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="3:3">
+    <row r="294" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C294" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="3:3">
+    <row r="295" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C295" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="3:3">
+    <row r="296" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C296" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="3:3">
+    <row r="297" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C297" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="3:3">
+    <row r="298" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C298" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="3:3">
+    <row r="299" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C299" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="3:3">
+    <row r="300" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C300" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="3:3">
+    <row r="301" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C301" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="3:3">
+    <row r="302" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C302" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="3:3">
+    <row r="303" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C303" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="3:3">
+    <row r="304" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C304" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="3:3">
+    <row r="305" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C305" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="3:3">
+    <row r="306" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C306" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="3:3">
+    <row r="307" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C307" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="3:3">
+    <row r="308" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C308" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="3:3">
+    <row r="309" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C309" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="3:3">
+    <row r="310" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C310" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="3:3">
+    <row r="311" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C311" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="3:3">
+    <row r="312" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C312" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="3:3">
+    <row r="313" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C313" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="3:3">
+    <row r="314" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C314" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="3:3">
+    <row r="315" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C315" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="3:3">
+    <row r="316" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C316" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="3:3">
+    <row r="317" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C317" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="3:3">
+    <row r="318" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C318" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="3:3">
+    <row r="319" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C319" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="3:3">
+    <row r="320" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C320" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="3:3">
+    <row r="321" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C321" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="3:3">
+    <row r="322" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C322" s="2">
         <f t="shared" ref="C322:C345" si="6">A322-B322</f>
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="3:3">
+    <row r="323" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C323" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="3:3">
+    <row r="324" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C324" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="3:3">
+    <row r="325" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C325" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="3:3">
+    <row r="326" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C326" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="3:3">
+    <row r="327" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C327" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="328" spans="3:3">
+    <row r="328" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C328" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="3:3">
+    <row r="329" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C329" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="3:3">
+    <row r="330" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C330" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="3:3">
+    <row r="331" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C331" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="3:3">
+    <row r="332" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C332" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="3:3">
+    <row r="333" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C333" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="3:3">
+    <row r="334" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C334" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="335" spans="3:3">
+    <row r="335" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C335" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="336" spans="3:3">
+    <row r="336" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C336" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="3:3">
+    <row r="337" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C337" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="338" spans="3:3">
+    <row r="338" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C338" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="3:3">
+    <row r="339" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C339" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="340" spans="3:3">
+    <row r="340" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C340" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="341" spans="3:3">
+    <row r="341" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C341" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="3:3">
+    <row r="342" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C342" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="3:3">
+    <row r="343" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C343" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="3:3">
+    <row r="344" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C344" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="3:3">
+    <row r="345" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C345" s="2">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="180" verticalDpi="180"/>
-  <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ED96D2B-D060-4D19-83A0-06CFB9C06380}">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0.50655899999999998</v>
+      </c>
+      <c r="B2">
+        <v>0.70824399999999998</v>
+      </c>
+      <c r="C2">
+        <v>0.79736099999999999</v>
+      </c>
+      <c r="D2">
+        <v>0.93807099999999999</v>
+      </c>
+      <c r="E2">
+        <v>1.2148019999999999</v>
+      </c>
+      <c r="F2">
+        <v>1.355513</v>
+      </c>
+      <c r="G2">
+        <v>1.6181730000000001</v>
+      </c>
+      <c r="H2">
+        <v>1.984021</v>
+      </c>
+      <c r="I2">
+        <v>1.9136660000000001</v>
+      </c>
+      <c r="J2">
+        <v>2.0731380000000001</v>
+      </c>
+      <c r="K2">
+        <v>2.134112</v>
+      </c>
+      <c r="L2">
+        <v>2.4155340000000001</v>
+      </c>
+      <c r="M2">
+        <v>2.504651</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0.55346200000000001</v>
+      </c>
+      <c r="B3">
+        <v>0.65664999999999996</v>
+      </c>
+      <c r="C3">
+        <v>0.81612200000000001</v>
+      </c>
+      <c r="D3">
+        <v>0.95683300000000004</v>
+      </c>
+      <c r="E3">
+        <v>1.18197</v>
+      </c>
+      <c r="F3">
+        <v>1.3132999999999999</v>
+      </c>
+      <c r="G3">
+        <v>1.7025999999999999</v>
+      </c>
+      <c r="H3">
+        <v>1.9699500000000001</v>
+      </c>
+      <c r="I3">
+        <v>1.923046</v>
+      </c>
+      <c r="J3">
+        <v>2.021544</v>
+      </c>
+      <c r="K3">
+        <v>2.1106609999999999</v>
+      </c>
+      <c r="L3">
+        <v>2.4577469999999999</v>
+      </c>
+      <c r="M3">
+        <v>2.5281020000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0.52063000000000004</v>
+      </c>
+      <c r="B4">
+        <v>0.70355400000000001</v>
+      </c>
+      <c r="C4">
+        <v>0.81143200000000004</v>
+      </c>
+      <c r="D4">
+        <v>0.91930999999999996</v>
+      </c>
+      <c r="E4">
+        <v>1.1772800000000001</v>
+      </c>
+      <c r="F4">
+        <v>1.341442</v>
+      </c>
+      <c r="G4">
+        <v>1.608792</v>
+      </c>
+      <c r="H4">
+        <v>1.941808</v>
+      </c>
+      <c r="I4">
+        <v>1.8995949999999999</v>
+      </c>
+      <c r="J4">
+        <v>2.10128</v>
+      </c>
+      <c r="K4">
+        <v>2.10128</v>
+      </c>
+      <c r="L4">
+        <v>2.4202240000000002</v>
+      </c>
+      <c r="M4">
+        <v>2.523412</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0.54877200000000004</v>
+      </c>
+      <c r="B5">
+        <v>0.68479199999999996</v>
+      </c>
+      <c r="C5">
+        <v>0.80674100000000004</v>
+      </c>
+      <c r="D5">
+        <v>0.97559399999999996</v>
+      </c>
+      <c r="E5">
+        <v>1.2101120000000001</v>
+      </c>
+      <c r="F5">
+        <v>1.322681</v>
+      </c>
+      <c r="G5">
+        <v>1.6228640000000001</v>
+      </c>
+      <c r="H5">
+        <v>1.937117</v>
+      </c>
+      <c r="I5">
+        <v>1.937117</v>
+      </c>
+      <c r="J5">
+        <v>2.0262340000000001</v>
+      </c>
+      <c r="K5">
+        <v>2.09659</v>
+      </c>
+      <c r="L5">
+        <v>2.4249149999999999</v>
+      </c>
+      <c r="M5">
+        <v>2.4858889999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0.51124899999999995</v>
+      </c>
+      <c r="B6">
+        <v>0.72231500000000004</v>
+      </c>
+      <c r="C6">
+        <v>0.82081199999999999</v>
+      </c>
+      <c r="D6">
+        <v>0.94745199999999996</v>
+      </c>
+      <c r="E6">
+        <v>1.224183</v>
+      </c>
+      <c r="F6">
+        <v>1.3695839999999999</v>
+      </c>
+      <c r="G6">
+        <v>1.6556960000000001</v>
+      </c>
+      <c r="H6">
+        <v>2.0027819999999998</v>
+      </c>
+      <c r="I6">
+        <v>1.9136660000000001</v>
+      </c>
+      <c r="J6">
+        <v>1.97464</v>
+      </c>
+      <c r="K6">
+        <v>2.1434929999999999</v>
+      </c>
+      <c r="L6">
+        <v>2.3639399999999999</v>
+      </c>
+      <c r="M6">
+        <v>2.5374829999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0.50655899999999998</v>
+      </c>
+      <c r="B7">
+        <v>0.69886300000000001</v>
+      </c>
+      <c r="C7">
+        <v>0.80205099999999996</v>
+      </c>
+      <c r="D7">
+        <v>0.98966500000000002</v>
+      </c>
+      <c r="E7">
+        <v>1.2288730000000001</v>
+      </c>
+      <c r="F7">
+        <v>1.3039190000000001</v>
+      </c>
+      <c r="G7">
+        <v>1.6603859999999999</v>
+      </c>
+      <c r="H7">
+        <v>1.979331</v>
+      </c>
+      <c r="I7">
+        <v>1.8902140000000001</v>
+      </c>
+      <c r="J7">
+        <v>2.0309249999999999</v>
+      </c>
+      <c r="K7">
+        <v>2.115351</v>
+      </c>
+      <c r="L7">
+        <v>2.3967719999999999</v>
+      </c>
+      <c r="M7">
+        <v>2.4999600000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0.52532000000000001</v>
+      </c>
+      <c r="B8">
+        <v>0.65664999999999996</v>
+      </c>
+      <c r="C8">
+        <v>0.82081199999999999</v>
+      </c>
+      <c r="D8">
+        <v>0.95683300000000004</v>
+      </c>
+      <c r="E8">
+        <v>1.205422</v>
+      </c>
+      <c r="F8">
+        <v>1.299229</v>
+      </c>
+      <c r="G8">
+        <v>1.6275539999999999</v>
+      </c>
+      <c r="H8">
+        <v>1.941808</v>
+      </c>
+      <c r="I8">
+        <v>1.9089750000000001</v>
+      </c>
+      <c r="J8">
+        <v>2.0449959999999998</v>
+      </c>
+      <c r="K8">
+        <v>2.10128</v>
+      </c>
+      <c r="L8">
+        <v>2.4155340000000001</v>
+      </c>
+      <c r="M8">
+        <v>2.4952700000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0.58160400000000001</v>
+      </c>
+      <c r="B9">
+        <v>0.68010199999999998</v>
+      </c>
+      <c r="C9">
+        <v>0.80674100000000004</v>
+      </c>
+      <c r="D9">
+        <v>0.93338100000000002</v>
+      </c>
+      <c r="E9">
+        <v>1.2523249999999999</v>
+      </c>
+      <c r="F9">
+        <v>1.3132999999999999</v>
+      </c>
+      <c r="G9">
+        <v>1.6181730000000001</v>
+      </c>
+      <c r="H9">
+        <v>1.998092</v>
+      </c>
+      <c r="I9">
+        <v>1.8995949999999999</v>
+      </c>
+      <c r="J9">
+        <v>2.0121630000000001</v>
+      </c>
+      <c r="K9">
+        <v>2.1388029999999998</v>
+      </c>
+      <c r="L9">
+        <v>2.382701</v>
+      </c>
+      <c r="M9">
+        <v>2.5281020000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0.55815300000000001</v>
+      </c>
+      <c r="B10">
+        <v>0.71293399999999996</v>
+      </c>
+      <c r="C10">
+        <v>0.83488399999999996</v>
+      </c>
+      <c r="D10">
+        <v>0.90054900000000004</v>
+      </c>
+      <c r="E10">
+        <v>1.2101120000000001</v>
+      </c>
+      <c r="F10">
+        <v>1.2663960000000001</v>
+      </c>
+      <c r="G10">
+        <v>1.651006</v>
+      </c>
+      <c r="H10">
+        <v>1.9558789999999999</v>
+      </c>
+      <c r="I10">
+        <v>1.8949039999999999</v>
+      </c>
+      <c r="J10">
+        <v>2.0168539999999999</v>
+      </c>
+      <c r="K10">
+        <v>2.0825179999999999</v>
+      </c>
+      <c r="L10">
+        <v>2.429605</v>
+      </c>
+      <c r="M10">
+        <v>2.5374819999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0.53470099999999998</v>
+      </c>
+      <c r="B11">
+        <v>0.68948200000000004</v>
+      </c>
+      <c r="C11">
+        <v>0.81143200000000004</v>
+      </c>
+      <c r="D11">
+        <v>0.91930999999999996</v>
+      </c>
+      <c r="E11">
+        <v>1.1585179999999999</v>
+      </c>
+      <c r="F11">
+        <v>1.341442</v>
+      </c>
+      <c r="G11">
+        <v>1.669767</v>
+      </c>
+      <c r="H11">
+        <v>1.9464980000000001</v>
+      </c>
+      <c r="I11">
+        <v>1.918356</v>
+      </c>
+      <c r="J11">
+        <v>2.054376</v>
+      </c>
+      <c r="K11">
+        <v>2.1106609999999999</v>
+      </c>
+      <c r="L11">
+        <v>2.3967719999999999</v>
+      </c>
+      <c r="M11">
+        <v>2.4718179999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <f>AVERAGE(A2:A11)</f>
+        <v>0.53470089999999992</v>
+      </c>
+      <c r="B13">
+        <f t="shared" ref="B13:M13" si="0">AVERAGE(B2:B11)</f>
+        <v>0.69135859999999993</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>0.81283879999999997</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>0.94369979999999987</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>1.2063597000000001</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>1.3226806000000002</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>1.6435011000000004</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>1.9657285999999998</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="0"/>
+        <v>1.9099134</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>2.035615</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="0"/>
+        <v>2.1134748999999999</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>2.4103743999999998</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="0"/>
+        <v>2.5112169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <f>A13*1000</f>
+        <v>534.70089999999993</v>
+      </c>
+      <c r="B14">
+        <f t="shared" ref="B14:M14" si="1">B13*1000</f>
+        <v>691.35859999999991</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="1"/>
+        <v>812.83879999999999</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="1"/>
+        <v>943.69979999999987</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="1"/>
+        <v>1206.3597000000002</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>1322.6806000000001</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>1643.5011000000004</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>1965.7285999999999</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="1"/>
+        <v>1909.9133999999999</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="1"/>
+        <v>2035.615</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="1"/>
+        <v>2113.4749000000002</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="1"/>
+        <v>2410.3743999999997</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="1"/>
+        <v>2511.2168999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>